<commit_message>
Cite the dairy and brewery models by their authors
The dairy files no longer cite a student data set (its student authors
and repository link): the stream data are credited to the DWSIM dairy
model of Bhatnagar, Flórez-Orrego, Boztas and Dardor and to the ROSMOSE
paper of Dardor, Flórez-Orrego et al. (2024), cited separately. The
brewery model is cited as the manuscript of Bhatnagar, Flórez-Orrego et
al., its DWSIM model credited to Bhatnagar, Flórez-Orrego and Boztas,
without the link to the student repository; the manuscript moves into
the references of the brewery case studies. Applied to the case studies,
data workbooks, course files, dairy Lua headers, JSON and pages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3-IndustrialProcesses/FoodAndBeverage/Dairy/Documents/DairyBiog_V3_rs_qt.xlsx
+++ b/3-IndustrialProcesses/FoodAndBeverage/Dairy/Documents/DairyBiog_V3_rs_qt.xlsx
@@ -51,7 +51,7 @@
     <t xml:space="preserve">t/h</t>
   </si>
   <si>
-    <t xml:space="preserve">IPESE dairy model (Dardor et al., 2024)</t>
+    <t xml:space="preserve">DWSIM dairy model of Bhatnagar, Flórez-Orrego, Boztas and Dardor; Dardor et al. (2024)</t>
   </si>
   <si>
     <t xml:space="preserve">Operating time</t>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Basis of all tables</t>
   </si>
   <si>
-    <t xml:space="preserve">Data: IPESE dairy model (DWSIM simulation implemented in ROSMOSE), latest MER runs; IETS Task XXIV dairy data set.</t>
+    <t xml:space="preserve">Data: DWSIM dairy model of Bhatnagar, Flórez-Orrego, Boztas and Dardor; Dardor et al. (2024); latest MER runs.</t>
   </si>
   <si>
     <t xml:space="preserve">Evaporator described effect by effect; condensing and boiling streams use dTmin/2 = 2 K, liquid streams 5 K.</t>

</xml_diff>